<commit_message>
Working With Properties and Excel Reading and DataProvider
</commit_message>
<xml_diff>
--- a/src/test/resources/excelData/TestData.xlsx
+++ b/src/test/resources/excelData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/19dcebdf543d4f4e/Desktop/May2026/Selenium_Jun_2026/LearningSelenium/src/test/resources/excelData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{669EAD17-0A0B-4D33-881B-A4EF3DDFFB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{669EAD17-0A0B-4D33-881B-A4EF3DDFFB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF30019-AE5C-437C-ADA5-821A7BBFC6FF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{263F8A78-6C45-4A09-846F-4C27EEBFAF9D}"/>
   </bookViews>
@@ -27,32 +27,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>testing123</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>password1</t>
   </si>
   <si>
-    <t>testing456</t>
-  </si>
-  <si>
     <t>password2</t>
   </si>
   <si>
-    <t>testing890</t>
-  </si>
-  <si>
     <t>password3</t>
+  </si>
+  <si>
+    <t>usernamepassword</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>username1</t>
+  </si>
+  <si>
+    <t>username2</t>
+  </si>
+  <si>
+    <t>username3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -80,8 +94,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,31 +413,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D755919C-03F2-4E22-91AB-833A1B03F294}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="9.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>